<commit_message>
chore: promote Pal Eyes R9.0.1 governed baseline
</commit_message>
<xml_diff>
--- a/data/trackers/PAL_EYES_MASTER_SITE_STATUS_TRACKER_CURRENT.xlsx
+++ b/data/trackers/PAL_EYES_MASTER_SITE_STATUS_TRACKER_CURRENT.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb2335e69b8124950"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sites" sheetId="2" r:id="Rb8edbabf45a04259"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Rb776ec89b5534780"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Editorial" sheetId="4" r:id="R071c9f77968d4dff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Held Claims" sheetId="5" r:id="Re3f8f086fca64b7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relations" sheetId="6" r:id="R0fe62138109b4766"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coordinates" sheetId="7" r:id="R3ac075cd6c224b59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="8" r:id="Rf52d2f9307a24ae8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UAT Contract" sheetId="9" r:id="R1d3dff39c6f64550"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Original Draft Layer" sheetId="10" r:id="R4c0664a3cb2643f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operational Backend" sheetId="11" r:id="R0b5fffb5bcae472e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R9e0a4bbacc264efe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sites" sheetId="2" r:id="Rceabf1ae235f4805"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R94073270c0de48c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Editorial" sheetId="4" r:id="R0a39917000554659"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Held Claims" sheetId="5" r:id="R7af4d91861df4123"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relations" sheetId="6" r:id="R471c010437d94665"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coordinates" sheetId="7" r:id="R9a8d022e076844b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="8" r:id="R85ee5c0659f14721"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UAT Contract" sheetId="9" r:id="R50fbc857a5994671"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Original Draft Layer" sheetId="10" r:id="Rec4f32a4e6004095"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operational Backend" sheetId="11" r:id="Rc3af3fe9bfa3400b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23,7 +23,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="4">
+  <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -46,8 +46,14 @@
       <x:color rgb="FF17202A"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF17212B"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="16">
+  <x:fills count="18">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -124,6 +130,16 @@
         <x:fgColor rgb="FF12304A"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B2742"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE9D4A7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -132,7 +148,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="87">
+  <x:cellXfs count="95">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -361,6 +377,26 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -721,7 +757,7 @@
   <x:cols>
     <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="48" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="43" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
@@ -731,7 +767,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>بعيون فلسطينية — Governed Content Adoption R5.1.0</x:v>
+        <x:v>بعيون فلسطينية — Direct Flutter Public Experience R9.0.0</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -778,7 +814,7 @@
         <x:v>Target Baseline</x:v>
       </x:c>
       <x:c r="E5" s="21" t="str">
-        <x:v>PAL_EYES_PUBLIC_EXPERIENCE_ATLAS_MUSEUM_MAGAZINE_R8_0_1_20260720</x:v>
+        <x:v>PAL_EYES_DIRECT_FLUTTER_PUBLIC_EXPERIENCE_MATURITY_R9_0_0_20260802</x:v>
       </x:c>
       <x:c r="F5" s="21" t="str"/>
       <x:c r="G5" s="21" t="str"/>
@@ -796,7 +832,7 @@
         <x:v>Implementation</x:v>
       </x:c>
       <x:c r="E6" s="21" t="str">
-        <x:v>BUILT_PENDING_LOCAL_UAT_R8_0_1</x:v>
+        <x:v>BUILT_PENDING_LOCAL_UAT_R9_0_0</x:v>
       </x:c>
       <x:c r="F6" s="21" t="str"/>
       <x:c r="G6" s="21" t="str"/>
@@ -875,7 +911,7 @@
         <x:v>Next Gate</x:v>
       </x:c>
       <x:c r="E10" s="21" t="str">
-        <x:v>Apply R8.0.1 and repeat analyzer/test before browser UAT</x:v>
+        <x:v>Apply R9.0.0, format/analyze/test, then desktop/mobile browser UAT</x:v>
       </x:c>
       <x:c r="F10" s="21" t="str"/>
       <x:c r="G10" s="21" t="str"/>
@@ -1587,6 +1623,192 @@
       <x:c r="D76" s="20" t="str">
         <x:v>No write; release blocked</x:v>
       </x:c>
+    </x:row>
+    <x:row r="78" ht="24" customHeight="1">
+      <x:c r="A78" s="91" t="str">
+        <x:v>R8.0.2 runtime closure</x:v>
+      </x:c>
+      <x:c r="B78" s="91" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="C78" s="91" t="str">
+        <x:v>Evidence</x:v>
+      </x:c>
+      <x:c r="D78" s="91"/>
+    </x:row>
+    <x:row r="79" ht="24" customHeight="1">
+      <x:c r="A79" s="20" t="str">
+        <x:v>Apply / static</x:v>
+      </x:c>
+      <x:c r="B79" s="20" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="C79" s="20" t="str">
+        <x:v>Bounded media stage</x:v>
+      </x:c>
+      <x:c r="D79" s="20"/>
+    </x:row>
+    <x:row r="80" ht="24" customHeight="1">
+      <x:c r="A80" s="20" t="str">
+        <x:v>Flutter analyze</x:v>
+      </x:c>
+      <x:c r="B80" s="20" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="C80" s="20" t="str">
+        <x:v>No issues found</x:v>
+      </x:c>
+      <x:c r="D80" s="20"/>
+    </x:row>
+    <x:row r="81" ht="24" customHeight="1">
+      <x:c r="A81" s="20" t="str">
+        <x:v>Flutter test</x:v>
+      </x:c>
+      <x:c r="B81" s="20" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="C81" s="20" t="str">
+        <x:v>58 tests</x:v>
+      </x:c>
+      <x:c r="D81" s="20"/>
+    </x:row>
+    <x:row r="82" ht="24" customHeight="1">
+      <x:c r="A82" s="20" t="str">
+        <x:v>Browser runtime smoke</x:v>
+      </x:c>
+      <x:c r="B82" s="20" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="C82" s="20" t="str">
+        <x:v>No Stack cascade</x:v>
+      </x:c>
+      <x:c r="D82" s="20"/>
+    </x:row>
+    <x:row r="83" ht="24" customHeight="1">
+      <x:c r="A83" s="20" t="str">
+        <x:v>Visual UAT</x:v>
+      </x:c>
+      <x:c r="B83" s="20" t="str">
+        <x:v>PENDING</x:v>
+      </x:c>
+      <x:c r="C83" s="20" t="str">
+        <x:v>Desktop + mobile</x:v>
+      </x:c>
+      <x:c r="D83" s="20"/>
+    </x:row>
+    <x:row r="84" ht="24" customHeight="1">
+      <x:c r="A84" s="20"/>
+      <x:c r="B84" s="20"/>
+      <x:c r="C84" s="20"/>
+      <x:c r="D84" s="20"/>
+    </x:row>
+    <x:row r="85" ht="24" customHeight="1">
+      <x:c r="A85" s="91" t="str">
+        <x:v>R9.0.0 direct Flutter maturity</x:v>
+      </x:c>
+      <x:c r="B85" s="91" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="C85" s="91" t="str">
+        <x:v>Evidence</x:v>
+      </x:c>
+      <x:c r="D85" s="91"/>
+    </x:row>
+    <x:row r="86" ht="24" customHeight="1">
+      <x:c r="A86" s="20" t="str">
+        <x:v>Figma workflow</x:v>
+      </x:c>
+      <x:c r="B86" s="20" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="C86" s="20" t="str">
+        <x:v>Structure preserved</x:v>
+      </x:c>
+      <x:c r="D86" s="20"/>
+    </x:row>
+    <x:row r="87" ht="24" customHeight="1">
+      <x:c r="A87" s="20" t="str">
+        <x:v>Public identity</x:v>
+      </x:c>
+      <x:c r="B87" s="20" t="str">
+        <x:v>BUILT</x:v>
+      </x:c>
+      <x:c r="C87" s="20" t="str">
+        <x:v>Atlas + Museum + Magazine</x:v>
+      </x:c>
+      <x:c r="D87" s="20"/>
+    </x:row>
+    <x:row r="88" ht="24" customHeight="1">
+      <x:c r="A88" s="20" t="str">
+        <x:v>Atlas / magazine preludes</x:v>
+      </x:c>
+      <x:c r="B88" s="20" t="str">
+        <x:v>BUILT</x:v>
+      </x:c>
+      <x:c r="C88" s="20" t="str">
+        <x:v>Editorial metrics + journeys</x:v>
+      </x:c>
+      <x:c r="D88" s="20"/>
+    </x:row>
+    <x:row r="89" ht="24" customHeight="1">
+      <x:c r="A89" s="20" t="str">
+        <x:v>Place detail</x:v>
+      </x:c>
+      <x:c r="B89" s="20" t="str">
+        <x:v>BUILT</x:v>
+      </x:c>
+      <x:c r="C89" s="20" t="str">
+        <x:v>Accessible content compass</x:v>
+      </x:c>
+      <x:c r="D89" s="20"/>
+    </x:row>
+    <x:row r="90" ht="24" customHeight="1">
+      <x:c r="A90" s="20" t="str">
+        <x:v>Story detail</x:v>
+      </x:c>
+      <x:c r="B90" s="20" t="str">
+        <x:v>BUILT</x:v>
+      </x:c>
+      <x:c r="C90" s="20" t="str">
+        <x:v>Chapter rail + reading frame</x:v>
+      </x:c>
+      <x:c r="D90" s="20"/>
+    </x:row>
+    <x:row r="91" ht="24" customHeight="1">
+      <x:c r="A91" s="20" t="str">
+        <x:v>Map zero-coordinate state</x:v>
+      </x:c>
+      <x:c r="B91" s="20" t="str">
+        <x:v>BUILT</x:v>
+      </x:c>
+      <x:c r="C91" s="20" t="str">
+        <x:v>Useful fail-closed gateway</x:v>
+      </x:c>
+      <x:c r="D91" s="20"/>
+    </x:row>
+    <x:row r="92" ht="24" customHeight="1">
+      <x:c r="A92" s="20" t="str">
+        <x:v>390px RTL tests</x:v>
+      </x:c>
+      <x:c r="B92" s="20" t="str">
+        <x:v>ADDED</x:v>
+      </x:c>
+      <x:c r="C92" s="20" t="str">
+        <x:v>No exception contract</x:v>
+      </x:c>
+      <x:c r="D92" s="20"/>
+    </x:row>
+    <x:row r="93" ht="24" customHeight="1">
+      <x:c r="A93" s="20" t="str">
+        <x:v>Database / publication</x:v>
+      </x:c>
+      <x:c r="B93" s="20" t="str">
+        <x:v>BLOCKED</x:v>
+      </x:c>
+      <x:c r="C93" s="20" t="str">
+        <x:v>No write; no release</x:v>
+      </x:c>
+      <x:c r="D93" s="20"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4489,10 +4711,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC2" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD2" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE2" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -4594,10 +4816,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC3" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD3" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE3" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -4701,10 +4923,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC4" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD4" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE4" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -4800,10 +5022,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC5" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD5" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE5" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -4901,10 +5123,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC6" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD6" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE6" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -5002,10 +5224,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC7" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD7" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE7" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -5107,10 +5329,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC8" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD8" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE8" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -5210,10 +5432,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC9" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD9" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE9" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -5313,10 +5535,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC10" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD10" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE10" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -5418,10 +5640,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC11" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD11" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE11" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -5523,10 +5745,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC12" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD12" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE12" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -5624,10 +5846,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC13" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD13" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE13" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -5723,10 +5945,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC14" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD14" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE14" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -5828,10 +6050,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC15" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD15" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE15" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -5929,10 +6151,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC16" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD16" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE16" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -6032,10 +6254,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC17" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD17" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE17" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -6133,10 +6355,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC18" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD18" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE18" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -6232,10 +6454,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC19" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD19" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE19" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -6337,10 +6559,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC20" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD20" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE20" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -6440,10 +6662,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC21" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD21" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE21" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -6541,10 +6763,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC22" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD22" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE22" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -6646,10 +6868,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC23" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD23" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE23" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -6747,10 +6969,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC24" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD24" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE24" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -6848,10 +7070,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC25" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD25" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE25" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -6949,10 +7171,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC26" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD26" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE26" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -7054,10 +7276,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC27" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD27" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE27" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -7157,10 +7379,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC28" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD28" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE28" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -7260,10 +7482,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC29" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD29" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE29" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -7361,10 +7583,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC30" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD30" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE30" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -7466,10 +7688,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC31" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD31" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE31" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -7571,10 +7793,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC32" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD32" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE32" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -7676,10 +7898,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC33" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD33" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE33" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -7777,10 +7999,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC34" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD34" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE34" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -7876,10 +8098,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC35" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD35" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE35" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -7977,10 +8199,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC36" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD36" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE36" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -8084,10 +8306,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC37" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD37" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE37" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -8189,10 +8411,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC38" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD38" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE38" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -8290,10 +8512,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC39" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD39" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE39" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -8397,10 +8619,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC40" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD40" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE40" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -8500,10 +8722,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC41" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD41" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE41" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -8605,10 +8827,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC42" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD42" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE42" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -8710,10 +8932,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC43" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD43" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE43" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -8811,10 +9033,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC44" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD44" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE44" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -8914,10 +9136,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC45" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD45" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE45" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -9013,10 +9235,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC46" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD46" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE46" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -9116,10 +9338,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC47" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD47" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE47" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -9217,10 +9439,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC48" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD48" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE48" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -9316,10 +9538,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC49" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD49" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE49" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -9415,10 +9637,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC50" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD50" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE50" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -9514,10 +9736,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC51" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD51" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE51" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -9613,10 +9835,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC52" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD52" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE52" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -9714,10 +9936,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC53" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD53" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE53" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -9813,10 +10035,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC54" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD54" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE54" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -9912,10 +10134,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC55" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD55" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE55" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -10011,10 +10233,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC56" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD56" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE56" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -10110,10 +10332,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC57" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD57" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE57" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -10211,10 +10433,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC58" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD58" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE58" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -10312,10 +10534,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC59" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD59" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE59" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -10413,10 +10635,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC60" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD60" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE60" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -10518,10 +10740,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC61" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD61" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE61" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -10617,10 +10839,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC62" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD62" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE62" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -10718,10 +10940,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC63" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD63" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE63" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -10823,10 +11045,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC64" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD64" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE64" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -10924,10 +11146,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC65" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD65" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE65" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -11027,10 +11249,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC66" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD66" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE66" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -11130,10 +11352,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC67" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD67" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE67" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -11233,10 +11455,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC68" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD68" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE68" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -11334,10 +11556,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC69" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD69" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE69" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -11441,10 +11663,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC70" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD70" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE70" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -11548,10 +11770,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC71" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD71" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE71" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -11653,10 +11875,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC72" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD72" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE72" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -11758,10 +11980,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC73" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD73" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE73" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -11865,10 +12087,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC74" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD74" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE74" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -11970,10 +12192,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC75" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD75" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE75" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -12077,10 +12299,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC76" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD76" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE76" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -12180,10 +12402,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC77" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD77" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE77" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -12285,10 +12507,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC78" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD78" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE78" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -12392,10 +12614,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC79" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD79" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE79" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -12499,10 +12721,10 @@
         <x:v>NO_APPROVED_MEDIA_ASSET</x:v>
       </x:c>
       <x:c r="AC80" s="21" t="str">
-        <x:v>IMPLEMENTED_PENDING_LOCAL_UAT</x:v>
+        <x:v>R9_0_0_UI_BUILT_PENDING_LOCAL_UAT</x:v>
       </x:c>
       <x:c r="AD80" s="21" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="AE80" s="21" t="str">
         <x:v>BLOCKED</x:v>
@@ -12547,7 +12769,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc2adb9a366f434d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc29cad3f6264d3d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16799,7 +17021,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc490f1c79244ef9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57d614d09a534ae9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20079,7 +20301,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0da5b4952874481c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7c4136f5e7a4b94"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29435,7 +29657,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e6b57545dc54b70"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4743598fc8b448ed"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29810,7 +30032,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0686deb12304332"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93401077193b450a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31849,7 +32071,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5de604bd23514611"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbceffbf0f862419c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32103,10 +32325,61 @@
         <x:v>USER_GOVERNING_DECISION_20260715</x:v>
       </x:c>
     </x:row>
+    <x:row r="15" ht="36" customHeight="1">
+      <x:c r="A15" s="20" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+      <x:c r="B15" s="20" t="str">
+        <x:v>R8_0_2_MEDIA_STAGE_RUNTIME_CLOSURE</x:v>
+      </x:c>
+      <x:c r="C15" s="20" t="str">
+        <x:v>PASS_RUNTIME_SMOKE_VISUAL_UAT_PENDING</x:v>
+      </x:c>
+      <x:c r="D15" s="20" t="str">
+        <x:v>إغلاق Stack غير محدود ونجاح الفاحص وAnalyzer و58 اختباراً وتشغيل Chrome دون عودة الانهيار.</x:v>
+      </x:c>
+      <x:c r="E15" s="20" t="str">
+        <x:v>PAL_EYES_PUBLIC_EXPERIENCE_MEDIA_STAGE_BOUNDED_LAYOUT_R8_0_2_20260802</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="36" customHeight="1">
+      <x:c r="A16" s="20" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+      <x:c r="B16" s="20" t="str">
+        <x:v>FIGMA_TRANSLATION_EXPERIMENT</x:v>
+      </x:c>
+      <x:c r="C16" s="20" t="str">
+        <x:v>CLOSED_NON_AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="D16" s="20" t="str">
+        <x:v>حفظ بنية Figma وإلغاء صفتها الإلزامية لأن واجهات Flutter المقبولة أقوى بصرياً.</x:v>
+      </x:c>
+      <x:c r="E16" s="20" t="str">
+        <x:v>MEGA_BATCH_PAL_EYES_FIGMA_DESIGN_SYSTEM_AND_PUBLIC_EXPERIENCE_TRANSLATION_V1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="36" customHeight="1">
+      <x:c r="A17" s="20" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+      <x:c r="B17" s="20" t="str">
+        <x:v>DIRECT_FLUTTER_PUBLIC_EXPERIENCE_R9</x:v>
+      </x:c>
+      <x:c r="C17" s="20" t="str">
+        <x:v>BUILT_PENDING_LOCAL_UAT</x:v>
+      </x:c>
+      <x:c r="D17" s="20" t="str">
+        <x:v>هوية أطلس/متحف/مجلة وافتتاحيات تحريرية وبوصلة محتوى ودليل فصول وتجربة خريطة fail-closed مفيدة.</x:v>
+      </x:c>
+      <x:c r="E17" s="20" t="str">
+        <x:v>PAL_EYES_DIRECT_FLUTTER_PUBLIC_EXPERIENCE_MATURITY_R9_0_0_20260802</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra302ff431c2a40af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R591463265e1a4344"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33119,6 +33392,162 @@
       </x:c>
       <x:c r="D88" s="20" t="str"/>
     </x:row>
+    <x:row r="90" ht="30" customHeight="1">
+      <x:c r="A90" s="94" t="str">
+        <x:v>R8.0.2 runtime smoke</x:v>
+      </x:c>
+      <x:c r="B90" s="94" t="str">
+        <x:v>No Stack size.isFinite cascade</x:v>
+      </x:c>
+      <x:c r="C90" s="94" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="D90" s="94"/>
+    </x:row>
+    <x:row r="91" ht="30" customHeight="1">
+      <x:c r="A91" s="20" t="str">
+        <x:v>R9.0.0 WhatIf</x:v>
+      </x:c>
+      <x:c r="B91" s="20" t="str">
+        <x:v>Source contract passes</x:v>
+      </x:c>
+      <x:c r="C91" s="20" t="str">
+        <x:v>READY</x:v>
+      </x:c>
+      <x:c r="D91" s="20"/>
+    </x:row>
+    <x:row r="92" ht="30" customHeight="1">
+      <x:c r="A92" s="20" t="str">
+        <x:v>R9.0.0 static</x:v>
+      </x:c>
+      <x:c r="B92" s="20" t="str">
+        <x:v>All direct Flutter maturity checks PASS</x:v>
+      </x:c>
+      <x:c r="C92" s="20" t="str">
+        <x:v>READY</x:v>
+      </x:c>
+      <x:c r="D92" s="20"/>
+    </x:row>
+    <x:row r="93" ht="30" customHeight="1">
+      <x:c r="A93" s="20" t="str">
+        <x:v>R9 widget tests</x:v>
+      </x:c>
+      <x:c r="B93" s="20" t="str">
+        <x:v>390px RTL + desktop adaptation + no exception</x:v>
+      </x:c>
+      <x:c r="C93" s="20" t="str">
+        <x:v>READY</x:v>
+      </x:c>
+      <x:c r="D93" s="20"/>
+    </x:row>
+    <x:row r="94" ht="30" customHeight="1">
+      <x:c r="A94" s="20" t="str">
+        <x:v>Flutter analyze</x:v>
+      </x:c>
+      <x:c r="B94" s="20" t="str">
+        <x:v>No issues found</x:v>
+      </x:c>
+      <x:c r="C94" s="20" t="str">
+        <x:v>PENDING_LOCAL</x:v>
+      </x:c>
+      <x:c r="D94" s="20"/>
+    </x:row>
+    <x:row r="95" ht="30" customHeight="1">
+      <x:c r="A95" s="20" t="str">
+        <x:v>Flutter test</x:v>
+      </x:c>
+      <x:c r="B95" s="20" t="str">
+        <x:v>All tests passed</x:v>
+      </x:c>
+      <x:c r="C95" s="20" t="str">
+        <x:v>PENDING_LOCAL</x:v>
+      </x:c>
+      <x:c r="D95" s="20"/>
+    </x:row>
+    <x:row r="96" ht="30" customHeight="1">
+      <x:c r="A96" s="20" t="str">
+        <x:v>Desktop visual UAT</x:v>
+      </x:c>
+      <x:c r="B96" s="20" t="str">
+        <x:v>Atlas / museum / magazine hierarchy</x:v>
+      </x:c>
+      <x:c r="C96" s="20" t="str">
+        <x:v>PENDING_LOCAL</x:v>
+      </x:c>
+      <x:c r="D96" s="20"/>
+    </x:row>
+    <x:row r="97" ht="30" customHeight="1">
+      <x:c r="A97" s="20" t="str">
+        <x:v>Mobile visual UAT</x:v>
+      </x:c>
+      <x:c r="B97" s="20" t="str">
+        <x:v>390x844, no clipping or overflow</x:v>
+      </x:c>
+      <x:c r="C97" s="20" t="str">
+        <x:v>PENDING_LOCAL</x:v>
+      </x:c>
+      <x:c r="D97" s="20"/>
+    </x:row>
+    <x:row r="98" ht="30" customHeight="1">
+      <x:c r="A98" s="20" t="str">
+        <x:v>RTL UAT</x:v>
+      </x:c>
+      <x:c r="B98" s="20" t="str">
+        <x:v>Direction, icons, navigation and reading order</x:v>
+      </x:c>
+      <x:c r="C98" s="20" t="str">
+        <x:v>PENDING_LOCAL</x:v>
+      </x:c>
+      <x:c r="D98" s="20"/>
+    </x:row>
+    <x:row r="99" ht="30" customHeight="1">
+      <x:c r="A99" s="20" t="str">
+        <x:v>Accessibility UAT</x:v>
+      </x:c>
+      <x:c r="B99" s="20" t="str">
+        <x:v>Focus, keyboard, 125% and 150% zoom</x:v>
+      </x:c>
+      <x:c r="C99" s="20" t="str">
+        <x:v>PENDING_LOCAL</x:v>
+      </x:c>
+      <x:c r="D99" s="20"/>
+    </x:row>
+    <x:row r="100" ht="30" customHeight="1">
+      <x:c r="A100" s="20" t="str">
+        <x:v>Runtime exceptions</x:v>
+      </x:c>
+      <x:c r="B100" s="20" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C100" s="20" t="str">
+        <x:v>PENDING_LOCAL</x:v>
+      </x:c>
+      <x:c r="D100" s="20"/>
+    </x:row>
+    <x:row r="101" ht="30" customHeight="1">
+      <x:c r="A101" s="20" t="str">
+        <x:v>Render overflows</x:v>
+      </x:c>
+      <x:c r="B101" s="20" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C101" s="20" t="str">
+        <x:v>PENDING_LOCAL</x:v>
+      </x:c>
+      <x:c r="D101" s="20"/>
+    </x:row>
+    <x:row r="102" ht="30" customHeight="1">
+      <x:c r="A102" s="20" t="str">
+        <x:v>Database / publication</x:v>
+      </x:c>
+      <x:c r="B102" s="20" t="str">
+        <x:v>No write; no release</x:v>
+      </x:c>
+      <x:c r="C102" s="20" t="str">
+        <x:v>BLOCKED</x:v>
+      </x:c>
+      <x:c r="D102" s="20"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>